<commit_message>
Fix tutorial exit flow and refresh POG art
This patch keeps the tutorial marked incomplete when a player exits early, preventing it from auto-starting again on a new game while still allowing replay from the main menu. It also updates the power-up icon resources to use the new POG art assets and refreshes the exit-warning copy and tutorial test expectations to match the intended behavior.
</commit_message>
<xml_diff>
--- a/Docs/powerup_registry_icons_updated.xlsx
+++ b/Docs/powerup_registry_icons_updated.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30527"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\danie\Documents\dicerogue\DiceRogue\Docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0A152C9E-F999-4529-BDF5-925C11BF2C5D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3FD0446B-814E-45FD-B3AA-484A2B0BF677}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1128,6 +1128,20 @@
   </cellStyles>
   <dxfs count="3">
     <dxf>
+      <border outline="0">
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <bottom style="thin">
+          <color auto="1"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
       <font>
         <b/>
         <i val="0"/>
@@ -1156,20 +1170,6 @@
         <bottom/>
       </border>
     </dxf>
-    <dxf>
-      <border outline="0">
-        <bottom style="thin">
-          <color auto="1"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border outline="0">
-        <top style="thin">
-          <color auto="1"/>
-        </top>
-      </border>
-    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -1184,7 +1184,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{B3CBC14D-CAA2-484C-88D5-95B1D618ECF4}" name="Table1" displayName="Table1" ref="A1:H73" totalsRowShown="0" headerRowDxfId="0" headerRowBorderDxfId="1" tableBorderDxfId="2">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{B3CBC14D-CAA2-484C-88D5-95B1D618ECF4}" name="Table1" displayName="Table1" ref="A1:H73" totalsRowShown="0" headerRowDxfId="2" headerRowBorderDxfId="1" tableBorderDxfId="0">
   <autoFilter ref="A1:H73" xr:uid="{B3CBC14D-CAA2-484C-88D5-95B1D618ECF4}"/>
   <tableColumns count="8">
     <tableColumn id="1" xr3:uid="{E896B0EC-B11D-4360-8FD2-38AF43B57F57}" name="file"/>
@@ -1677,7 +1677,7 @@
         <v>278</v>
       </c>
       <c r="H7" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.35">
@@ -1703,7 +1703,7 @@
         <v>279</v>
       </c>
       <c r="H8" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.35">
@@ -1729,7 +1729,7 @@
         <v>280</v>
       </c>
       <c r="H9" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.35">
@@ -1755,7 +1755,7 @@
         <v>281</v>
       </c>
       <c r="H10" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.35">

</xml_diff>